<commit_message>
chore: atualiza OSG TOTAL.xlsx
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/OSG TOTAL.xlsx
+++ b/OSG TOTAL.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\DEPARTAMENTO DE ESTUDOS E PLANEJAMENTO ORÇAMENTARIO\LUISA_ESTUDOS E MONITORAMENTO\Relatório OSG_Luísa\Banco de Dados OSG\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\icaro.lebre\Documents\Temáticos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C69F86D8-9D0E-4306-BAD3-A2C654C7B357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8982AFEA-934B-4D0B-89FD-029F8F243EB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{A28D029C-85C5-43CB-BED4-18AB3696A19E}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{A28D029C-85C5-43CB-BED4-18AB3696A19E}"/>
   </bookViews>
   <sheets>
     <sheet name="CATEGORIA 1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2139" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2139" uniqueCount="391">
   <si>
     <t>Órgão</t>
   </si>
@@ -1203,6 +1203,9 @@
   </si>
   <si>
     <t>VALORIZAÇÃO E CAPACITAÇÃO DOS SERVIDORES DA SEOP.</t>
+  </si>
+  <si>
+    <t>Orçamento Atualizado</t>
   </si>
 </sst>
 </file>
@@ -8122,7 +8125,7 @@
         <v>4</v>
       </c>
       <c r="L2" s="38" t="s">
-        <v>63</v>
+        <v>390</v>
       </c>
       <c r="M2" s="5" t="s">
         <v>64</v>

</xml_diff>